<commit_message>
Initial commit: QuickStay backend, frontend, Docker, CI, QA
</commit_message>
<xml_diff>
--- a/docs/QuickStay-Calendar.xlsx
+++ b/docs/QuickStay-Calendar.xlsx
@@ -189,6 +189,160 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
+      <t xml:space="preserve">• T027 docker-compose: dịch vụ mysql có healthchec…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T030 Tạo PR template và quy ước commit
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T233 Soạn .gitignore và cấu trúc thư mục repo (b…
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F6FB5"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Hưng (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T016 Viết SRS 2.1–2.2: sơ đồ quan hệ đối tượng v…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T017 Viết SRS 2.3–2.4: sơ đồ luồng và sơ đồ chuy…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T018 Viết SRS 2.5–2.6: phân quyền chức năng, dữ …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T019 Họp daily, cập nhật bảng công việc
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF3D8B37"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Vượng (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T020 Viết entity User, UserRepository và tài kho…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T021 API đăng ký: validate dữ liệu, chuẩn hóa em…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T022 API đăng nhập và sinh JWT có hạn (JwtServic…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD96A1B"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Đức (6.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T023 Wireframe dashboard admin: 3 tab Đặt phòng,…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T024 Wireframe chatbot và bản mobile
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T025 Khởi tạo React + Vite + Tailwind + Zustand …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T026 Dựng layout chung và khung Navbar
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7030A0"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Minh (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
       <t xml:space="preserve">• T014 Viết Dockerfile backend (Gradle + JDK)
 </t>
     </r>
@@ -197,9 +351,179 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
+      <t xml:space="preserve">• T041 GitHub Actions: build và test backend khi p…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T234 Viết nginx.conf: proxy /api sang backend và…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T235 README khung: giới thiệu, công nghệ, cấu tr…
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F6FB5"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Hưng (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T031 Đặc tả use case UC06 (đặt phòng) trong SRS
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T032 Đặc tả use case UC12 (sinh mô tả AI) trong …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T033 Đặc tả use case UC13 (chatbot) trong SRS
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T034 Viết test case UC01–UC03 (mã, bước, kết quả…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF3D8B37"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Vượng (7 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T035 Unit test API đăng ký (thành công, trùng em…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T037 Viết seed dữ liệu mẫu 4 khách sạn và các lo…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T036 Viết entity Hotel, Room, Booking và reposit…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD96A1B"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Đức (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T038 Giao diện trang Đăng nhập
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T039 Giao diện trang Đăng ký
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T040 Viết authStore (Zustand) và hàm gọi API tự …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7030A0"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Minh (7 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T043 Spring Security: JwtAuthFilter và cấu hình …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
       <t xml:space="preserve">• T015 Viết Dockerfile frontend (Node build + Ngin…
 </t>
     </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T028 docker-compose: backend, frontend, biến môi…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T029 Viết README hướng dẫn chạy dự án
+</t>
+    </r>
   </si>
   <si>
     <r>
@@ -217,31 +541,31 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T016 Viết SRS 2.1–2.2: sơ đồ quan hệ đối tượng v…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T017 Viết SRS 2.3–2.4: sơ đồ luồng và sơ đồ chuy…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T018 Viết SRS 2.5–2.6: phân quyền chức năng, dữ …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T019 Họp daily, cập nhật bảng công việc
+      <t xml:space="preserve">• T044 Viết test case UC04–UC05 (tìm kiếm, phòng t…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T045 Viết test case UC06–UC08 (đặt phòng, lịch s…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T046 Viết test case UC09–UC13 (admin, AI)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T047 Họp daily, cập nhật bảng công việc
 </t>
     </r>
     <r>
@@ -259,23 +583,23 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T020 Viết entity User, UserRepository và tài kho…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T021 API đăng ký: validate dữ liệu, chuẩn hóa em…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T022 API đăng nhập và sinh JWT có hạn (JwtServic…
+      <t xml:space="preserve">• T048 API danh sách khách sạn kèm giá thấp nhất m…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T049 Tìm kiếm theo tên hoặc thành phố (khớp một …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T050 Lọc theo loại phòng và khoảng giá
 </t>
     </r>
     <r>
@@ -285,39 +609,31 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Đức (6.5 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T023 Wireframe dashboard admin: 3 tab Đặt phòng,…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T024 Wireframe chatbot và bản mobile
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T025 Khởi tạo React + Vite + Tailwind + Zustand …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T026 Dựng layout chung và khung Navbar
+      <t xml:space="preserve">Đức (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T051 Nối API đăng nhập, đăng ký và hiển thị lỗi …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T052 Navbar theo vai trò và route guard (CUSTOME…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T053 Trang chủ: lưới thẻ khách sạn (ảnh, tên, th…
 </t>
     </r>
     <r>
@@ -335,31 +651,31 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T027 docker-compose: dịch vụ mysql có healthchec…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T028 docker-compose: backend, frontend, biến môi…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T029 Viết README hướng dẫn chạy dự án
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T030 Tạo PR template và quy ước commit
+      <t xml:space="preserve">• T054 Cấu hình CORS chỉ cho nguồn Frontend
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T055 Xử lý 401 và 403 trả JSON (accessDeniedHand…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T056 Viết test phân quyền qua HTTP thật (TestRes…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T057 Đặc tả use case UC09–UC11 (quản trị) trong …
 </t>
     </r>
   </si>
@@ -379,31 +695,31 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T031 Đặc tả use case UC06 (đặt phòng) trong SRS
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T032 Đặc tả use case UC12 (sinh mô tả AI) trong …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T033 Đặc tả use case UC13 (chatbot) trong SRS
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T034 Viết test case UC01–UC03 (mã, bước, kết quả…
+      <t xml:space="preserve">• T058 Viết SRS phần 4: component, thông báo, cảnh…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T059 Kiểm thử thủ công đăng ký, đăng nhập; ghi l…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T060 Review PR tuần 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T061 Sprint Review và Retro tuần 1
 </t>
     </r>
     <r>
@@ -421,23 +737,23 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T035 Unit test API đăng ký (thành công, trùng em…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T036 Viết entity Hotel, Room và repository
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T037 Viết seed dữ liệu mẫu 4 khách sạn và các lo…
+      <t xml:space="preserve">• T062 API chi tiết một khách sạn (GET /hotels/{id…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T063 Unit test tìm kiếm và lọc khách sạn
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T064 API xem và cập nhật hồ sơ (GET/PUT /users/m…
 </t>
     </r>
     <r>
@@ -455,23 +771,31 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T038 Giao diện trang Đăng nhập
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T039 Giao diện trang Đăng ký
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T040 Viết authStore (Zustand) và hàm gọi API tự …
+      <t xml:space="preserve">• T065 Trang chủ: ô tìm kiếm theo tên/thành phố và…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T066 Trang chủ: bộ lọc loại phòng và khoảng giá
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T067 Trang chủ: trạng thái đang tải, rỗng, lỗi
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T068 Sprint Review và Retro tuần 1
 </t>
     </r>
     <r>
@@ -481,15 +805,23 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T041 GitHub Actions: build và test backend khi p…
+      <t xml:space="preserve">Minh (6.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T070 Chạy thử toàn hệ thống bằng docker compose …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T072 Sprint Review và Retro tuần 1
 </t>
     </r>
     <r>
@@ -505,323 +837,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T043 Spring Security: JwtAuthFilter và cấu hình …
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F6FB5"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Hưng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T044 Viết test case UC04–UC05 (tìm kiếm, phòng t…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T045 Viết test case UC06–UC08 (đặt phòng, lịch s…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T046 Viết test case UC09–UC13 (admin, AI)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T047 Họp daily, cập nhật bảng công việc
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF3D8B37"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Vượng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T048 API danh sách khách sạn kèm giá thấp nhất m…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T049 Tìm kiếm theo tên hoặc thành phố (khớp một …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T050 Lọc theo loại phòng và khoảng giá
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD96A1B"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Đức (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T051 Nối API đăng nhập, đăng ký và hiển thị lỗi …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T052 Navbar theo vai trò và route guard (CUSTOME…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T053 Trang chủ: lưới thẻ khách sạn (ảnh, tên, th…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7030A0"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T054 Cấu hình CORS chỉ cho nguồn Frontend
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T055 Xử lý 401 và 403 trả JSON (accessDeniedHand…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T056 Viết test phân quyền qua HTTP thật (TestRes…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T057 Đặc tả use case UC09–UC11 (quản trị) trong …
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F6FB5"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Hưng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T058 Viết SRS phần 4: component, thông báo, cảnh…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T059 Kiểm thử thủ công đăng ký, đăng nhập; ghi l…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T060 Review PR tuần 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T061 Sprint Review và Retro tuần 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF3D8B37"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Vượng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T062 API chi tiết một khách sạn (GET /hotels/{id…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T063 Unit test tìm kiếm và lọc khách sạn
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T064 API xem và cập nhật hồ sơ (GET/PUT /users/m…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD96A1B"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Đức (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T065 Trang chủ: ô tìm kiếm theo tên/thành phố và…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T066 Trang chủ: bộ lọc loại phòng và khoảng giá
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T067 Trang chủ: trạng thái đang tải, rỗng, lỗi
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T068 Sprint Review và Retro tuần 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7030A0"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T069 Rà soát bảo mật cấu hình: secret, biến môi …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T070 Chạy thử toàn hệ thống bằng docker compose …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T071 Logging SLF4J/Logback cho exception quan tr…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T072 Sprint Review và Retro tuần 1
+      <t xml:space="preserve">• T119 Bộ xử lý lỗi chung: trả {"message"} thống n…
 </t>
     </r>
   </si>
@@ -1384,15 +1400,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T119 Bộ xử lý lỗi chung: trả {"message"} thống n…
+      <t xml:space="preserve">Minh (7 giờ)
 </t>
     </r>
     <r>
@@ -1409,6 +1417,22 @@
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">• T121 Workflow đẩy Docker image lên GHCR khi push…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T069 Rà soát bảo mật cấu hình: secret, biến môi …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T071 Logging SLF4J/Logback cho exception quan tr…
 </t>
     </r>
   </si>
@@ -1598,6 +1622,282 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
+      <t xml:space="preserve">Hưng (6.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T136 Nút "Tạo mô tả bằng AI" ở form khách sạn
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T139 Thử AI thật với khóa API (nếu có) và ghi kế…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T148 Widget chatbot: nút tròn và khung chat
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF3D8B37"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Vượng (5.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T140 Bổ sung test: đăng ký, đăng nhập, hồ sơ (nh…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T142 Đo độ phủ test và liệt kê phần chưa phủ
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T165 API phân trang danh sách khách sạn và đơn đ…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD96A1B"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Đức (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T143 Admin tab Khách sạn: bảng danh sách và form…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T144 Admin tab Khách sạn: xóa, hộp thoại xác nhậ…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7030A0"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Minh (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T145 Triển khai: cài Docker và docker compose tr…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T146 Triển khai: Nginx reverse proxy và biến môi…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T147 Kiểm tra backup và khôi phục volume MySQL
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F6FB5"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Hưng (5.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T149 Widget chatbot: nối API, hiển thị tin nhắn,…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T150 Review PR
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T137 Nút "Tạo mô tả bằng AI" ở form phòng
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T138 Kiểm thử thủ công sinh mô tả AI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF3D8B37"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Vượng (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T151 Bổ sung test: đặt phòng, lịch sử, hủy (nhán…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T152 Bổ sung test: API admin và phân quyền
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T153 Tối ưu truy vấn phòng trống và thêm chỉ mục…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD96A1B"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Đức (7.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T154 Admin tab Phòng: bảng danh sách và form thê…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T155 Admin tab Phòng: kiểm tra giá, sức chứa, số…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T236 Giao diện phân trang danh sách khách sạn và…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7030A0"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Minh (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T156 Smoke test toàn bộ luồng trên môi trường tr…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T157 Rà soát bảo mật: CORS, secret, log không lộ…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T158 Chuẩn bị merge dev vào main, giải quyết xun…
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F6FB5"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
       <t xml:space="preserve">Hưng (6 giờ)
 </t>
     </r>
@@ -1606,31 +1906,39 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T136 Nút "Tạo mô tả bằng AI" ở form khách sạn
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T137 Nút "Tạo mô tả bằng AI" ở form phòng
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T138 Kiểm thử thủ công sinh mô tả AI
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T139 Thử AI thật với khóa API (nếu có) và ghi kế…
+      <t xml:space="preserve">• T159 Chạy E2E toàn luồng trên bản docker compose
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T160 Kiểm thử tải 50 request đồng thời
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T161 Đo Lighthouse (First Contentful Paint)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T162 Khóa tính năng mới lúc 12h; từ đó chỉ sửa l…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T163 Review PR
 </t>
     </r>
     <r>
@@ -1640,6 +1948,136 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
+      <t xml:space="preserve">Vượng (6.5 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T164 Test đồng thời chống đặt trùng: nhiều yêu c…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T166 Sửa lỗi QA phía backend
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T141 Bổ sung test: khách sạn, tìm kiếm, phòng tr…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD96A1B"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Đức (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T167 Responsive Trang chủ và Chi tiết khách sạn …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T168 Responsive Đặt phòng, Lịch sử, Hồ sơ, Đăng …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7030A0"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Minh (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T169 Pipeline CI xanh trên nhánh dev
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T170 Merge dev vào main sau khi review
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T171 Đẩy Docker image lên GHCR từ main
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F6FB5"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Hưng (6 giờ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T172 Báo cáo kiểm thử: tổng hợp số liệu test và …
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T173 Đóng các lỗi còn lại trong cột Bug cùng ngư…
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T174 Rà soát lịch sử commit của 4 thành viên
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF3D8B37"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+      </rPr>
       <t xml:space="preserve">Vượng (6 giờ)
 </t>
     </r>
@@ -1648,420 +2086,6 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">• T140 Bổ sung test: đăng ký, đăng nhập, hồ sơ (nh…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T141 Bổ sung test: khách sạn, tìm kiếm, phòng tr…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T142 Đo độ phủ test và liệt kê phần chưa phủ
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD96A1B"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Đức (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T143 Admin tab Khách sạn: bảng danh sách và form…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T144 Admin tab Khách sạn: xóa, hộp thoại xác nhậ…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7030A0"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T145 Triển khai: cài Docker và docker compose tr…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T146 Triển khai: Nginx reverse proxy và biến môi…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T147 Kiểm tra backup và khôi phục volume MySQL
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F6FB5"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Hưng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T148 Widget chatbot: nút tròn và khung chat
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T149 Widget chatbot: nối API, hiển thị tin nhắn,…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T150 Review PR
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF3D8B37"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Vượng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T151 Bổ sung test: đặt phòng, lịch sử, hủy (nhán…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T152 Bổ sung test: API admin và phân quyền
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T153 Tối ưu truy vấn phòng trống và thêm chỉ mục…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD96A1B"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Đức (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T154 Admin tab Phòng: bảng danh sách và form thê…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T155 Admin tab Phòng: kiểm tra giá, sức chứa, số…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7030A0"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T156 Smoke test toàn bộ luồng trên môi trường tr…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T157 Rà soát bảo mật: CORS, secret, log không lộ…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T158 Chuẩn bị merge dev vào main, giải quyết xun…
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F6FB5"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Hưng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T159 Chạy E2E toàn luồng trên bản docker compose
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T160 Kiểm thử tải 50 request đồng thời
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T161 Đo Lighthouse (First Contentful Paint)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T162 Khóa tính năng mới lúc 12h; từ đó chỉ sửa l…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T163 Review PR
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF3D8B37"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Vượng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T164 Test đồng thời chống đặt trùng: nhiều yêu c…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T165 API phân trang danh sách khách sạn và đơn đ…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T166 Sửa lỗi QA phía backend
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD96A1B"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Đức (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T167 Responsive Trang chủ và Chi tiết khách sạn …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T168 Responsive Đặt phòng, Lịch sử, Hồ sơ, Đăng …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7030A0"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Minh (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T169 Pipeline CI xanh trên nhánh dev
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T170 Merge dev vào main sau khi review
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T171 Đẩy Docker image lên GHCR từ main
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F6FB5"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Hưng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T172 Báo cáo kiểm thử: tổng hợp số liệu test và …
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T173 Đóng các lỗi còn lại trong cột Bug cùng ngư…
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T174 Rà soát lịch sử commit của 4 thành viên
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF3D8B37"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Vượng (6 giờ)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">• T175 Hỗ trợ Đức nối API phân trang ở giao diện
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-      </rPr>
       <t xml:space="preserve">• T176 Sửa lỗi backend theo kết quả tải và Lightho…
 </t>
     </r>
@@ -2071,6 +2095,14 @@
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">• T177 Chốt tài liệu API và ERD theo thực tế
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">• T175 Kiểm thử phân trang qua API và giao diện, s…
 </t>
     </r>
     <r>

</xml_diff>